<commit_message>
Ui changed code altered
</commit_message>
<xml_diff>
--- a/mf_products_data.xlsx
+++ b/mf_products_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Suresh V\Desktop\automation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28719CE1-B1F6-4A2C-BA97-093F9AAB56E9}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08D85626-4F48-4572-A113-448FFDB2F846}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7950" yWindow="2595" windowWidth="17070" windowHeight="8205" activeTab="3" xr2:uid="{1E71232C-EF9C-4FE2-8681-349AE10419A2}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="13" activeTab="19" xr2:uid="{1E71232C-EF9C-4FE2-8681-349AE10419A2}"/>
   </bookViews>
   <sheets>
     <sheet name="category" sheetId="3" r:id="rId1"/>
@@ -23,19 +23,16 @@
     <sheet name="QR_Monitoring_Filters" sheetId="8" r:id="rId8"/>
     <sheet name="schedule_report_create" sheetId="15" r:id="rId9"/>
     <sheet name="schedule_report_filters" sheetId="16" r:id="rId10"/>
-    <sheet name="Sheet1" sheetId="17" r:id="rId11"/>
-    <sheet name="Sheet2" sheetId="18" r:id="rId12"/>
-    <sheet name="Sheet3" sheetId="19" r:id="rId13"/>
-    <sheet name="QR_Monitoring_Filter_By_field" sheetId="11" r:id="rId14"/>
-    <sheet name="QR_Monitoring_fake_product_fdb" sheetId="12" r:id="rId15"/>
-    <sheet name="QR_Monitoring_export_ID_based" sheetId="9" r:id="rId16"/>
-    <sheet name="QR_Monitoring_export_Bulk_ID" sheetId="10" r:id="rId17"/>
-    <sheet name="Batch_status_report" sheetId="13" r:id="rId18"/>
-    <sheet name="LoginData" sheetId="14" r:id="rId19"/>
-    <sheet name="Roles_and_permission_create" sheetId="20" r:id="rId20"/>
-    <sheet name="Roles_and_permission_filters" sheetId="21" r:id="rId21"/>
-    <sheet name="users_create" sheetId="22" r:id="rId22"/>
-    <sheet name="user_filters" sheetId="23" r:id="rId23"/>
+    <sheet name="QR_Monitoring_Filter_By_field" sheetId="11" r:id="rId11"/>
+    <sheet name="QR_Monitoring_fake_product_fdb" sheetId="12" r:id="rId12"/>
+    <sheet name="QR_Monitoring_export_ID_based" sheetId="9" r:id="rId13"/>
+    <sheet name="QR_Monitoring_export_Bulk_ID" sheetId="10" r:id="rId14"/>
+    <sheet name="Reports" sheetId="13" r:id="rId15"/>
+    <sheet name="LoginData" sheetId="14" r:id="rId16"/>
+    <sheet name="Roles_and_permission_create" sheetId="20" r:id="rId17"/>
+    <sheet name="Roles_and_permission_filters" sheetId="21" r:id="rId18"/>
+    <sheet name="users_create" sheetId="22" r:id="rId19"/>
+    <sheet name="user_filters" sheetId="23" r:id="rId20"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -47,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="179" uniqueCount="119">
   <si>
     <t>product_name</t>
   </si>
@@ -139,9 +136,6 @@
     <t>variants_value</t>
   </si>
   <si>
-    <t>002</t>
-  </si>
-  <si>
     <t>blue</t>
   </si>
   <si>
@@ -262,27 +256,12 @@
     <t>test</t>
   </si>
   <si>
-    <t>chair</t>
-  </si>
-  <si>
-    <t>plastic</t>
-  </si>
-  <si>
     <t>select_report</t>
   </si>
   <si>
     <t>mail_receiving_duration</t>
   </si>
   <si>
-    <t>Scan Analytics Report</t>
-  </si>
-  <si>
-    <t>Daily</t>
-  </si>
-  <si>
-    <t>11:00</t>
-  </si>
-  <si>
     <t>date_string</t>
   </si>
   <si>
@@ -301,18 +280,9 @@
     <t>Admin User - Manufacturer</t>
   </si>
   <si>
-    <t>poiuyq</t>
-  </si>
-  <si>
     <t>search_name</t>
   </si>
   <si>
-    <t>2026-02-01</t>
-  </si>
-  <si>
-    <t>2026-02-27</t>
-  </si>
-  <si>
     <t>user_name</t>
   </si>
   <si>
@@ -334,18 +304,9 @@
     <t>testing (Arihant)</t>
   </si>
   <si>
-    <t>abcd1234316790@gmail.com</t>
-  </si>
-  <si>
-    <t>demotest</t>
-  </si>
-  <si>
     <t>2026-03-01</t>
   </si>
   <si>
-    <t>2026-03-17</t>
-  </si>
-  <si>
     <t>QR_Type</t>
   </si>
   <si>
@@ -358,9 +319,6 @@
     <t>M155-MPGH-0087</t>
   </si>
   <si>
-    <t>PRD2025X0007</t>
-  </si>
-  <si>
     <t>B794-50</t>
   </si>
   <si>
@@ -373,10 +331,76 @@
     <t>2025-12-01</t>
   </si>
   <si>
-    <t>speakers</t>
-  </si>
-  <si>
-    <t>speakercovers</t>
+    <t>video_title</t>
+  </si>
+  <si>
+    <t>video_file</t>
+  </si>
+  <si>
+    <t xml:space="preserve">testing </t>
+  </si>
+  <si>
+    <t>C:\Users\Suresh V\Downloads\20260505_094627.mp4</t>
+  </si>
+  <si>
+    <t>testt</t>
+  </si>
+  <si>
+    <t>sheet</t>
+  </si>
+  <si>
+    <t>sheett</t>
+  </si>
+  <si>
+    <t>paper</t>
+  </si>
+  <si>
+    <t>paperr</t>
+  </si>
+  <si>
+    <t>mklp</t>
+  </si>
+  <si>
+    <t>mklpo</t>
+  </si>
+  <si>
+    <t>plasticssss</t>
+  </si>
+  <si>
+    <t>0024</t>
+  </si>
+  <si>
+    <t>PRD2026X00018</t>
+  </si>
+  <si>
+    <t>PRD2026X00019</t>
+  </si>
+  <si>
+    <t>Print Audit Report</t>
+  </si>
+  <si>
+    <t>16:00</t>
+  </si>
+  <si>
+    <t>Bi-Weekly</t>
+  </si>
+  <si>
+    <t>samples</t>
+  </si>
+  <si>
+    <t>demo</t>
+  </si>
+  <si>
+    <t>2026-05-06</t>
+  </si>
+  <si>
+    <t>2026-05-07</t>
+  </si>
+  <si>
+    <t>abcd12316790@gmail.com</t>
+  </si>
+  <si>
+    <t>2026-05-8</t>
   </si>
 </sst>
 </file>
@@ -526,9 +550,6 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -562,6 +583,9 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -880,7 +904,7 @@
   <dimension ref="A1:B3"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="14.42578125" customWidth="1"/>
+    <col min="1" max="1" width="31.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="15.75">
@@ -893,7 +917,7 @@
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="3" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="B2" s="7" t="s">
         <v>9</v>
@@ -901,9 +925,9 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" t="s">
-        <v>109</v>
-      </c>
-      <c r="B3" t="s">
+        <v>105</v>
+      </c>
+      <c r="B3" s="7" t="s">
         <v>9</v>
       </c>
     </row>
@@ -926,29 +950,29 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="B1" s="3" t="s">
         <v>55</v>
-      </c>
-      <c r="B1" s="3" t="s">
-        <v>56</v>
       </c>
       <c r="C1" s="3" t="s">
         <v>6</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>78</v>
+        <v>72</v>
       </c>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" s="3" t="s">
-        <v>80</v>
+        <v>74</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="C2" s="25" t="s">
-        <v>79</v>
-      </c>
-      <c r="D2" s="28">
+        <v>58</v>
+      </c>
+      <c r="C2" s="24" t="s">
+        <v>73</v>
+      </c>
+      <c r="D2" s="27">
         <v>46077</v>
       </c>
     </row>
@@ -983,33 +1007,6 @@
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{719DE049-13A9-41AD-8D77-209B4D420600}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{394B36C8-07D8-43F3-947E-E60737F16168}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{530E70C9-470C-48D5-826C-6E6296487FE3}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{805A6EDD-E425-4375-9798-049A39968A7E}">
   <dimension ref="A1:D5"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -1021,27 +1018,27 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4">
-      <c r="A1" s="19" t="s">
-        <v>32</v>
-      </c>
-      <c r="B1" s="19" t="s">
+      <c r="A1" s="18" t="s">
+        <v>31</v>
+      </c>
+      <c r="B1" s="18" t="s">
         <v>6</v>
       </c>
-      <c r="C1" s="19" t="s">
+      <c r="C1" s="18" t="s">
+        <v>42</v>
+      </c>
+      <c r="D1" s="18" t="s">
         <v>43</v>
-      </c>
-      <c r="D1" s="19" t="s">
-        <v>44</v>
       </c>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" s="3"/>
       <c r="B2" s="3"/>
-      <c r="C2" s="18" t="s">
-        <v>54</v>
-      </c>
-      <c r="D2" s="18" t="s">
-        <v>54</v>
+      <c r="C2" s="17" t="s">
+        <v>53</v>
+      </c>
+      <c r="D2" s="17" t="s">
+        <v>53</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -1068,7 +1065,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{28BF2E4E-D2AD-4788-84CE-589D65DD9913}">
   <dimension ref="A1:D4"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -1080,27 +1077,27 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4">
-      <c r="A1" s="19" t="s">
-        <v>32</v>
-      </c>
-      <c r="B1" s="19" t="s">
+      <c r="A1" s="18" t="s">
+        <v>31</v>
+      </c>
+      <c r="B1" s="18" t="s">
         <v>6</v>
       </c>
-      <c r="C1" s="19" t="s">
+      <c r="C1" s="18" t="s">
+        <v>42</v>
+      </c>
+      <c r="D1" s="18" t="s">
         <v>43</v>
-      </c>
-      <c r="D1" s="19" t="s">
-        <v>44</v>
       </c>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" s="3"/>
       <c r="B2" s="3"/>
-      <c r="C2" s="18" t="s">
-        <v>54</v>
-      </c>
-      <c r="D2" s="18" t="s">
-        <v>54</v>
+      <c r="C2" s="17" t="s">
+        <v>53</v>
+      </c>
+      <c r="D2" s="17" t="s">
+        <v>53</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -1120,7 +1117,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8C593467-91D7-45A0-AB4C-29552EB2F315}">
   <dimension ref="A1:C2"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -1132,13 +1129,13 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B1" t="s">
         <v>48</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>49</v>
-      </c>
-      <c r="C1" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="2" spans="1:3">
@@ -1149,7 +1146,7 @@
         <v>6000</v>
       </c>
       <c r="C2" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
   </sheetData>
@@ -1157,22 +1154,22 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DBE76918-F0A7-4D6C-A220-F9B93E3F4D71}">
   <dimension ref="A1:A3"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="19.7109375" style="14" customWidth="1"/>
+    <col min="1" max="1" width="19.7109375" style="13" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" s="4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="2" spans="1:1">
       <c r="A2" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="3" spans="1:1">
@@ -1184,7 +1181,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8812D42C-EE85-4119-BC63-85E0A2A59C8A}">
   <dimension ref="A1:C2"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -1195,25 +1192,25 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="19" t="s">
+        <v>54</v>
+      </c>
+      <c r="B1" t="s">
+        <v>56</v>
+      </c>
+      <c r="C1" t="s">
         <v>55</v>
-      </c>
-      <c r="B1" t="s">
-        <v>57</v>
-      </c>
-      <c r="C1" t="s">
-        <v>56</v>
       </c>
     </row>
     <row r="2" spans="1:3">
       <c r="A2" t="s">
+        <v>57</v>
+      </c>
+      <c r="B2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C2" t="s">
         <v>58</v>
-      </c>
-      <c r="B2" t="s">
-        <v>60</v>
-      </c>
-      <c r="C2" t="s">
-        <v>59</v>
       </c>
     </row>
   </sheetData>
@@ -1222,7 +1219,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7A9810B8-64D0-4E9C-8574-FE25F4330D20}">
   <dimension ref="A1:C4"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -1232,40 +1229,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" s="17" t="s">
-        <v>41</v>
-      </c>
-      <c r="B1" s="17" t="s">
-        <v>61</v>
-      </c>
-      <c r="C1" s="17" t="s">
-        <v>66</v>
+      <c r="A1" s="16" t="s">
+        <v>40</v>
+      </c>
+      <c r="B1" s="16" t="s">
+        <v>60</v>
+      </c>
+      <c r="C1" s="16" t="s">
+        <v>65</v>
       </c>
     </row>
     <row r="2" spans="1:3">
-      <c r="A2" s="21" t="s">
+      <c r="A2" s="20" t="s">
+        <v>63</v>
+      </c>
+      <c r="B2" s="5" t="s">
         <v>64</v>
-      </c>
-      <c r="B2" s="5" t="s">
-        <v>65</v>
       </c>
       <c r="C2" s="5"/>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="B3" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="B3" s="5" t="s">
-        <v>63</v>
-      </c>
       <c r="C3" s="5"/>
     </row>
     <row r="4" spans="1:3">
-      <c r="A4" s="24" t="s">
+      <c r="A4" s="23" t="s">
+        <v>67</v>
+      </c>
+      <c r="B4" s="23" t="s">
         <v>68</v>
-      </c>
-      <c r="B4" s="24" t="s">
-        <v>69</v>
       </c>
     </row>
   </sheetData>
@@ -1278,56 +1275,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{49965304-110C-43B7-8F15-D1A55CEFA51D}">
-  <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="27.28515625" customWidth="1"/>
-    <col min="2" max="2" width="17.140625" style="14" customWidth="1"/>
-    <col min="3" max="3" width="17.140625" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" ht="15.75">
-      <c r="A1" s="8" t="s">
-        <v>26</v>
-      </c>
-      <c r="B1" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="C1" s="8" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3">
-      <c r="A2" s="3" t="s">
-        <v>108</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3">
-      <c r="A3" t="s">
-        <v>109</v>
-      </c>
-      <c r="B3" s="14" t="s">
-        <v>30</v>
-      </c>
-      <c r="C3" t="s">
-        <v>31</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6F558A45-F57B-4E55-9D43-AC432A6721A1}">
   <dimension ref="A1:C6"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -1339,10 +1287,10 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" s="3" t="s">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="C1" s="3" t="s">
         <v>6</v>
@@ -1350,10 +1298,10 @@
     </row>
     <row r="2" spans="1:3">
       <c r="A2" s="3" t="s">
-        <v>96</v>
+        <v>113</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>9</v>
@@ -1385,7 +1333,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{43879EE9-C99F-4A5B-96F3-E1D0A9776555}">
   <dimension ref="A1:D5"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -1397,38 +1345,38 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4">
-      <c r="A1" s="19" t="s">
-        <v>85</v>
-      </c>
-      <c r="B1" s="19" t="s">
+      <c r="A1" s="18" t="s">
+        <v>78</v>
+      </c>
+      <c r="B1" s="18" t="s">
         <v>6</v>
       </c>
-      <c r="C1" s="19" t="s">
+      <c r="C1" s="18" t="s">
+        <v>42</v>
+      </c>
+      <c r="D1" s="18" t="s">
         <v>43</v>
       </c>
-      <c r="D1" s="19" t="s">
-        <v>44</v>
-      </c>
     </row>
     <row r="2" spans="1:4">
-      <c r="A2" s="16" t="s">
-        <v>84</v>
+      <c r="A2" s="15" t="s">
+        <v>114</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>79</v>
-      </c>
-      <c r="C2" s="18" t="s">
-        <v>86</v>
-      </c>
-      <c r="D2" s="18" t="s">
-        <v>87</v>
+        <v>73</v>
+      </c>
+      <c r="C2" s="17" t="s">
+        <v>115</v>
+      </c>
+      <c r="D2" s="17" t="s">
+        <v>116</v>
       </c>
     </row>
     <row r="3" spans="1:4">
-      <c r="A3" s="16"/>
+      <c r="A3" s="15"/>
       <c r="B3" s="3"/>
-      <c r="C3" s="18"/>
-      <c r="D3" s="18"/>
+      <c r="C3" s="17"/>
+      <c r="D3" s="17"/>
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="3"/>
@@ -1449,7 +1397,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D08D1696-D02C-4610-92E6-D56A7B92D2A5}">
   <dimension ref="A1:F7"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -1464,51 +1412,51 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="3" t="s">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="D1" s="3" t="s">
         <v>6</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>91</v>
+        <v>82</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="2" spans="1:6">
       <c r="A2" s="3" t="s">
-        <v>92</v>
+        <v>83</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>94</v>
-      </c>
-      <c r="C2" s="29" t="s">
-        <v>95</v>
+        <v>85</v>
+      </c>
+      <c r="C2" s="28" t="s">
+        <v>117</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E2" s="3">
-        <v>9876521895</v>
-      </c>
-      <c r="F2" s="29" t="s">
-        <v>93</v>
+        <v>9807521895</v>
+      </c>
+      <c r="F2" s="28" t="s">
+        <v>84</v>
       </c>
     </row>
     <row r="3" spans="1:6">
       <c r="A3" s="3"/>
       <c r="B3" s="3"/>
-      <c r="C3" s="29"/>
+      <c r="C3" s="28"/>
       <c r="D3" s="3"/>
       <c r="E3" s="3"/>
-      <c r="F3" s="29"/>
+      <c r="F3" s="28"/>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" s="3"/>
@@ -1552,7 +1500,56 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{49965304-110C-43B7-8F15-D1A55CEFA51D}">
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="27.28515625" customWidth="1"/>
+    <col min="2" max="2" width="17.140625" style="13" customWidth="1"/>
+    <col min="3" max="3" width="17.140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" ht="15.75">
+      <c r="A1" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="B1" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" t="s">
+        <v>101</v>
+      </c>
+      <c r="B3" s="13" t="s">
+        <v>107</v>
+      </c>
+      <c r="C3" t="s">
+        <v>30</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2E6FDA5E-64D6-4D8A-A7B1-583E8820775D}">
   <dimension ref="A1:D6"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -1564,31 +1561,31 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4">
-      <c r="A1" s="19" t="s">
-        <v>85</v>
-      </c>
-      <c r="B1" s="19" t="s">
+      <c r="A1" s="18" t="s">
+        <v>78</v>
+      </c>
+      <c r="B1" s="18" t="s">
         <v>6</v>
       </c>
-      <c r="C1" s="19" t="s">
+      <c r="C1" s="18" t="s">
+        <v>42</v>
+      </c>
+      <c r="D1" s="18" t="s">
         <v>43</v>
       </c>
-      <c r="D1" s="19" t="s">
-        <v>44</v>
-      </c>
     </row>
     <row r="2" spans="1:4">
-      <c r="A2" s="30" t="s">
-        <v>92</v>
+      <c r="A2" s="29" t="s">
+        <v>83</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>79</v>
-      </c>
-      <c r="C2" s="18" t="s">
-        <v>97</v>
-      </c>
-      <c r="D2" s="18" t="s">
-        <v>98</v>
+        <v>73</v>
+      </c>
+      <c r="C2" s="17" t="s">
+        <v>86</v>
+      </c>
+      <c r="D2" s="17" t="s">
+        <v>118</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -1633,8 +1630,8 @@
     <col min="7" max="7" width="16" customWidth="1"/>
     <col min="8" max="8" width="37.140625" customWidth="1"/>
     <col min="9" max="9" width="15.140625" customWidth="1"/>
-    <col min="10" max="10" width="14.5703125" customWidth="1"/>
-    <col min="11" max="11" width="20.42578125" customWidth="1"/>
+    <col min="10" max="10" width="20.42578125" customWidth="1"/>
+    <col min="11" max="11" width="53.28515625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="31.5">
@@ -1665,15 +1662,19 @@
       <c r="I1" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="10"/>
-      <c r="K1" s="10"/>
+      <c r="J1" s="10" t="s">
+        <v>95</v>
+      </c>
+      <c r="K1" s="30" t="s">
+        <v>96</v>
+      </c>
     </row>
     <row r="2" spans="1:11" ht="47.25">
       <c r="A2" s="11" t="s">
-        <v>108</v>
+        <v>102</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C2" s="11" t="s">
         <v>13</v>
@@ -1682,13 +1683,13 @@
         <v>14</v>
       </c>
       <c r="E2" s="11" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="F2" s="11" t="s">
         <v>9</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>71</v>
+        <v>100</v>
       </c>
       <c r="H2" s="11" t="s">
         <v>10</v>
@@ -1696,21 +1697,47 @@
       <c r="I2" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="J2" s="13"/>
-      <c r="K2" s="11"/>
-    </row>
-    <row r="3" spans="1:11" ht="15.75">
-      <c r="A3" s="11"/>
-      <c r="B3" s="11"/>
-      <c r="C3" s="11"/>
-      <c r="D3" s="12"/>
-      <c r="E3" s="11"/>
-      <c r="F3" s="11"/>
-      <c r="G3" s="3"/>
-      <c r="H3" s="11"/>
-      <c r="I3" s="11"/>
-      <c r="J3" s="13"/>
-      <c r="K3" s="11"/>
+      <c r="J2" s="11" t="s">
+        <v>97</v>
+      </c>
+      <c r="K2" s="3" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" ht="47.25">
+      <c r="A3" s="11" t="s">
+        <v>103</v>
+      </c>
+      <c r="B3" s="11" t="s">
+        <v>99</v>
+      </c>
+      <c r="C3" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="D3" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="E3" s="11" t="s">
+        <v>109</v>
+      </c>
+      <c r="F3" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="H3" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="I3" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="J3" s="11" t="s">
+        <v>97</v>
+      </c>
+      <c r="K3" s="3" t="s">
+        <v>98</v>
+      </c>
     </row>
     <row r="4" spans="1:11">
       <c r="A4" s="1"/>
@@ -1752,9 +1779,10 @@
   <phoneticPr fontId="2" type="noConversion"/>
   <hyperlinks>
     <hyperlink ref="D2" r:id="rId1" xr:uid="{8B51A6DA-AB47-4D21-B79F-C0F5CD9F6D1E}"/>
+    <hyperlink ref="D3" r:id="rId2" xr:uid="{7743F41D-75AB-44A3-B840-8FDE6759F018}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId2"/>
+  <pageSetup orientation="portrait" r:id="rId3"/>
 </worksheet>
 </file>
 
@@ -1800,16 +1828,16 @@
       <c r="H1" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="I1" s="22" t="s">
-        <v>99</v>
-      </c>
-      <c r="J1" s="22" t="s">
-        <v>101</v>
+      <c r="I1" s="21" t="s">
+        <v>87</v>
+      </c>
+      <c r="J1" s="21" t="s">
+        <v>89</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="30">
       <c r="A2" s="5" t="s">
-        <v>102</v>
+        <v>90</v>
       </c>
       <c r="B2" s="5">
         <v>1234</v>
@@ -1833,10 +1861,10 @@
         <v>24</v>
       </c>
       <c r="I2" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>100</v>
+        <v>88</v>
       </c>
     </row>
     <row r="3" spans="1:10">
@@ -1872,7 +1900,7 @@
       <c r="H5" s="1"/>
     </row>
     <row r="12" spans="1:10">
-      <c r="D12" s="23"/>
+      <c r="D12" s="22"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
@@ -1891,27 +1919,27 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
-      <c r="A1" s="15" t="s">
-        <v>32</v>
-      </c>
-      <c r="B1" s="15" t="s">
+      <c r="A1" s="14" t="s">
+        <v>31</v>
+      </c>
+      <c r="B1" s="14" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="3" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="3" t="s">
-        <v>104</v>
+        <v>91</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
   </sheetData>
@@ -1930,27 +1958,27 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
-      <c r="A1" s="15" t="s">
-        <v>32</v>
-      </c>
-      <c r="B1" s="15" t="s">
+      <c r="A1" s="14" t="s">
+        <v>31</v>
+      </c>
+      <c r="B1" s="14" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
   </sheetData>
@@ -1970,45 +1998,45 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="14" t="s">
+        <v>31</v>
+      </c>
+      <c r="B1" s="14" t="s">
+        <v>6</v>
+      </c>
+      <c r="C1" s="14" t="s">
+        <v>35</v>
+      </c>
+      <c r="D1" s="14" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="30">
+      <c r="A2" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="B1" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="C1" s="15" t="s">
+      <c r="C2" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="D1" s="15" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" ht="30">
-      <c r="A2" s="16" t="s">
+      <c r="D2" s="1" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="30">
+      <c r="A3" s="15" t="s">
         <v>38</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B3" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="C3" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="C2" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" ht="30">
-      <c r="A3" s="16" t="s">
+      <c r="D3" s="1" t="s">
         <v>39</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>40</v>
       </c>
     </row>
   </sheetData>
@@ -2030,47 +2058,47 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="17" t="s">
+      <c r="A1" s="16" t="s">
+        <v>40</v>
+      </c>
+      <c r="B1" s="16" t="s">
         <v>41</v>
       </c>
-      <c r="B1" s="17" t="s">
+      <c r="C1" s="16" t="s">
         <v>42</v>
       </c>
-      <c r="C1" s="17" t="s">
+      <c r="D1" s="16" t="s">
         <v>43</v>
       </c>
-      <c r="D1" s="17" t="s">
-        <v>44</v>
-      </c>
-      <c r="E1" s="15"/>
+      <c r="E1" s="14"/>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" s="5" t="s">
-        <v>105</v>
+        <v>92</v>
       </c>
       <c r="B2" s="5">
         <v>9619583752</v>
       </c>
-      <c r="C2" s="18" t="s">
-        <v>107</v>
-      </c>
-      <c r="D2" s="18" t="s">
-        <v>47</v>
+      <c r="C2" s="17" t="s">
+        <v>94</v>
+      </c>
+      <c r="D2" s="17" t="s">
+        <v>46</v>
       </c>
       <c r="E2" s="1"/>
     </row>
     <row r="3" spans="1:5">
       <c r="A3" s="5" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B3" s="5">
         <v>9999999999</v>
       </c>
-      <c r="C3" s="18" t="s">
-        <v>106</v>
-      </c>
-      <c r="D3" s="18" t="s">
-        <v>46</v>
+      <c r="C3" s="17" t="s">
+        <v>93</v>
+      </c>
+      <c r="D3" s="17" t="s">
+        <v>45</v>
       </c>
       <c r="E3" s="1"/>
     </row>
@@ -2089,7 +2117,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{47321248-6969-4F5E-944C-613388F81213}">
-  <dimension ref="A1:J16"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="28.7109375" customWidth="1"/>
@@ -2098,69 +2126,57 @@
     <col min="4" max="4" width="26" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10">
+    <row r="1" spans="1:5">
       <c r="A1" s="3" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="B1" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="C1" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="C1" s="3" t="s">
-        <v>57</v>
-      </c>
       <c r="D1" s="3" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="2" spans="1:10">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
       <c r="A2" s="3" t="s">
-        <v>75</v>
+        <v>110</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="C2" s="25" t="s">
-        <v>76</v>
-      </c>
-      <c r="D2" s="27" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10">
+        <v>58</v>
+      </c>
+      <c r="C2" s="24" t="s">
+        <v>112</v>
+      </c>
+      <c r="D2" s="26" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5">
       <c r="A3" s="3"/>
       <c r="B3" s="3"/>
       <c r="C3" s="3"/>
       <c r="D3" s="3"/>
-      <c r="J3" s="20"/>
-    </row>
-    <row r="4" spans="1:10">
+    </row>
+    <row r="4" spans="1:5">
       <c r="A4" s="3"/>
       <c r="B4" s="3"/>
       <c r="C4" s="3"/>
       <c r="D4" s="3"/>
     </row>
-    <row r="5" spans="1:10">
+    <row r="5" spans="1:5">
       <c r="A5" s="3"/>
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>
       <c r="D5" s="3"/>
     </row>
-    <row r="6" spans="1:10">
-      <c r="A6" s="3"/>
-      <c r="B6" s="3"/>
-      <c r="C6" s="3"/>
-      <c r="D6" s="3"/>
-    </row>
-    <row r="7" spans="1:10">
-      <c r="A7" s="3"/>
-      <c r="B7" s="3"/>
-      <c r="C7" s="3"/>
-      <c r="D7" s="3"/>
-    </row>
-    <row r="16" spans="1:10">
-      <c r="E16" s="26"/>
+    <row r="14" spans="1:5">
+      <c r="E14" s="25"/>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>